<commit_message>
Remove standalone FP Analysis and Entitlement Mapping tools
False-positive detection is now a toggle inside SOD & SA Analysis
(3-level FP pipeline in sod_sa_engine.py); entitlement mapping remains
only as an internal dependency of the ruleset mapping engine. Drop the
corresponding engines, routers, models, API clients, pages, and
templates, and move fp_database.xlsx under Data/SODSAAnalysis.

Also add the SOD & SA stress-data generator script and gitignore local
Claude settings, generated stress-test data, and local documentation.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/SODSAAnalysis/user_roles.xlsx
+++ b/Data/SODSAAnalysis/user_roles.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\khize\Study_Material\Projects\EY\Governance_Platform\Data\SODSAAnalysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{046638B6-13AF-40B2-9D5F-8261B67EBF03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEC287E1-EB0D-4592-9B23-583DD2237F6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="31">
   <si>
     <t>User Name</t>
   </si>
@@ -67,9 +67,6 @@
     <t>IT Administrator</t>
   </si>
   <si>
-    <t>bjones</t>
-  </si>
-  <si>
     <t>ROLE_FIN_DIRECTOR</t>
   </si>
   <si>
@@ -91,9 +88,6 @@
     <t>PO Clerk</t>
   </si>
   <si>
-    <t>epark</t>
-  </si>
-  <si>
     <t>ROLE_GL_ANALYST</t>
   </si>
   <si>
@@ -112,10 +106,13 @@
     <t>fsantos</t>
   </si>
   <si>
-    <t>jdoe adam sandler bullock</t>
-  </si>
-  <si>
-    <t>dkhan ibrahim Monday</t>
+    <t>dkhan ibrahim</t>
+  </si>
+  <si>
+    <t>jdoe adam</t>
+  </si>
+  <si>
+    <t>sandler bullock</t>
   </si>
 </sst>
 </file>
@@ -151,8 +148,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -455,158 +455,195 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B15" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C15" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C16" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>29</v>
-      </c>
-      <c r="B12" t="s">
-        <v>4</v>
-      </c>
-      <c r="C12" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C13" t="s">
-        <v>8</v>
-      </c>
-    </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C17">
+    <sortCondition ref="A2:A17"/>
+  </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>